<commit_message>
Add production Docker setup and dispatch log/UI polish
- New docker-compose.prod.yml: loopback-only port bindings, persistent
  media volume, no dev bind-mounts — built images are self-contained.
- New frontend/Dockerfile.prod + nginx.conf: real `vite build` served as
  static files via nginx-in-container, instead of the dev server.
- vite.config.js: allow arss.uz/www.arss.uz Host headers (Vite 5 rejects
  unrecognized hosts by default), needed behind the production reverse proxy.
- Add whitenoise so Django admin static files are actually served under
  gunicorn (DEBUG=False) instead of 404ing; entrypoint.sh runs collectstatic.
- Dispatch log Excel template: narrower Гуруҳ рақами/Машқ рақами/Ёқилғи/
  downtime columns per new column-width spec, with header label font size
  and row height adjusted so the narrower columns don't clip adjacent text.
- CarDetailView: margin between the Yo'l varaqasi and Tahrirlash buttons.
</commit_message>
<xml_diff>
--- a/backend/management/assets/dispatch_log_page_template.xlsx
+++ b/backend/management/assets/dispatch_log_page_template.xlsx
@@ -272,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -436,6 +436,15 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -805,18 +814,48 @@
   <dimension ref="A1:AP33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.515625" defaultRowHeight="14.25"/>
   <cols>
-    <col width="3.27" customWidth="1" min="1" max="1"/>
-    <col width="3.73" customWidth="1" min="7" max="7"/>
-    <col width="2.73" customWidth="1" min="8" max="8"/>
-    <col width="2.82" customWidth="1" min="9" max="9"/>
-    <col width="4" customWidth="1" min="10" max="10"/>
-    <col width="3.27" customWidth="1" min="11" max="11"/>
-    <col width="3.45" customWidth="1" min="12" max="12"/>
-    <col width="3.27" customWidth="1" min="13" max="13"/>
-    <col width="3.18" customWidth="1" min="19" max="19"/>
-    <col width="2.18" customWidth="1" min="40" max="40"/>
+    <col width="0.981" customWidth="1" min="1" max="1"/>
+    <col width="2.5547" customWidth="1" min="2" max="2"/>
+    <col width="2.5547" customWidth="1" min="3" max="3"/>
+    <col width="5.9609" customWidth="1" min="4" max="4"/>
+    <col width="5.9609" customWidth="1" min="5" max="5"/>
+    <col width="5.9609" customWidth="1" min="6" max="6"/>
+    <col width="2.611" customWidth="1" min="7" max="7"/>
+    <col width="1.911" customWidth="1" min="8" max="8"/>
+    <col width="1.974" customWidth="1" min="9" max="9"/>
+    <col width="2.8" customWidth="1" min="10" max="10"/>
+    <col width="2.289" customWidth="1" min="11" max="11"/>
+    <col width="2.415" customWidth="1" min="12" max="12"/>
+    <col width="2.289" customWidth="1" min="13" max="13"/>
+    <col width="5.9609" customWidth="1" min="14" max="14"/>
+    <col width="2.5547" customWidth="1" min="15" max="15"/>
+    <col width="2.5547" customWidth="1" min="16" max="16"/>
+    <col width="2.5547" customWidth="1" min="17" max="17"/>
+    <col width="4.2578" customWidth="1" min="18" max="18"/>
+    <col width="1.59" customWidth="1" min="19" max="19"/>
+    <col width="4.2578" customWidth="1" min="20" max="20"/>
+    <col width="4.2578" customWidth="1" min="21" max="21"/>
+    <col width="4.2578" customWidth="1" min="22" max="22"/>
+    <col width="4.2578" customWidth="1" min="23" max="23"/>
+    <col width="4.2578" customWidth="1" min="24" max="24"/>
+    <col width="4.2578" customWidth="1" min="25" max="25"/>
+    <col width="4.2578" customWidth="1" min="26" max="26"/>
+    <col width="4.2578" customWidth="1" min="27" max="27"/>
+    <col width="4.2578" customWidth="1" min="28" max="28"/>
+    <col width="4.2578" customWidth="1" min="29" max="29"/>
+    <col width="4.2578" customWidth="1" min="30" max="30"/>
+    <col width="4.2578" customWidth="1" min="31" max="31"/>
+    <col width="4.2578" customWidth="1" min="32" max="32"/>
+    <col width="4.2578" customWidth="1" min="33" max="33"/>
+    <col width="4.2578" customWidth="1" min="34" max="34"/>
+    <col width="4.2578" customWidth="1" min="35" max="35"/>
+    <col width="4.2578" customWidth="1" min="36" max="36"/>
+    <col width="4.2578" customWidth="1" min="37" max="37"/>
+    <col width="4.2578" customWidth="1" min="38" max="38"/>
+    <col width="4.2578" customWidth="1" min="39" max="39"/>
+    <col width="1.09" customWidth="1" min="40" max="40"/>
     <col width="3.18" customWidth="1" min="41" max="41"/>
-    <col width="4" customWidth="1" min="42" max="42"/>
+    <col width="2" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -923,7 +962,7 @@
       <c r="AJ7" s="11" t="n"/>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">Автомобил русуми </t>
         </is>
@@ -966,7 +1005,7 @@
       <c r="D9" s="11" t="n"/>
       <c r="E9" s="11" t="n"/>
       <c r="F9" s="11" t="n"/>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="61" t="inlineStr">
         <is>
           <t>Давлат рақами</t>
         </is>
@@ -1019,7 +1058,7 @@
       <c r="D10" s="11" t="n"/>
       <c r="E10" s="11" t="n"/>
       <c r="F10" s="11" t="n"/>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="G10" s="62" t="inlineStr">
         <is>
           <t>Уста</t>
         </is>
@@ -1257,7 +1296,7 @@
       <c r="AO19" s="19" t="n"/>
       <c r="AP19" s="31" t="n"/>
     </row>
-    <row r="20" ht="30.75" customHeight="1">
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
           <t>Гуруҳ рақами</t>
@@ -1855,7 +1894,6 @@
       <c r="AO31" s="19" t="n"/>
       <c r="AP31" s="31" t="n"/>
     </row>
-    <row r="32"/>
     <row r="33" ht="17.35" customHeight="1">
       <c r="C33" s="11" t="inlineStr">
         <is>
@@ -1888,8 +1926,8 @@
     <mergeCell ref="W26:Y26"/>
     <mergeCell ref="AD20:AK20"/>
     <mergeCell ref="AL27:AP27"/>
+    <mergeCell ref="AD23:AK23"/>
     <mergeCell ref="O25:Q25"/>
-    <mergeCell ref="AD23:AK23"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="D31:N31"/>
     <mergeCell ref="AL26:AP26"/>

</xml_diff>